<commit_message>
chore: master 覆盖为 codeBrave-World-node2 快照
按用户确认，将默认分支整树替换为功能分支快照（含 tslua2→Brave-World 改名）。
master 独有的 a55960d（技能特效/开发工具链/网关重构）内容被移除，但其提交仍保留在历史中，
可用 backup/master-before-overwrite 或 git revert 本提交恢复。
</commit_message>
<xml_diff>
--- a/tables/datas/__beans__.xlsx
+++ b/tables/datas/__beans__.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P98"/>
+  <dimension ref="A1:P103"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="20.625" customWidth="1" style="4" min="2" max="2"/>
@@ -810,6 +810,8 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15">
       <c r="B15" s="0" t="inlineStr">
         <is>
@@ -1059,6 +1061,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="B28" s="0" t="inlineStr">
         <is>
@@ -1884,34 +1887,34 @@
       </c>
     </row>
     <row r="70">
-      <c r="J70" t="inlineStr">
+      <c r="J70" s="0" t="inlineStr">
         <is>
           <t>projectile_speed</t>
         </is>
       </c>
-      <c r="L70" t="inlineStr">
+      <c r="L70" s="0" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr">
+      <c r="N70" s="0" t="inlineStr">
         <is>
           <t>弹道飞行速度(格/秒)</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="J71" t="inlineStr">
+      <c r="J71" s="0" t="inlineStr">
         <is>
           <t>projectile_max_range</t>
         </is>
       </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="N71" t="inlineStr">
+      <c r="L71" s="0" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="N71" s="0" t="inlineStr">
         <is>
           <t>弹道最大飞行距离(格)</t>
         </is>
@@ -2443,6 +2446,116 @@
       <c r="N98" s="0" t="inlineStr">
         <is>
           <t>掉落条目列表</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="J99" s="0" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="L99" s="0" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="M99" s="0" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="N99" s="0" t="inlineStr">
+        <is>
+          <t>章节标题</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="J100" s="0" t="inlineStr">
+        <is>
+          <t>chapter_id</t>
+        </is>
+      </c>
+      <c r="L100" s="0" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="M100" s="0" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="N100" s="0" t="inlineStr">
+        <is>
+          <t>所属章节ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="J101" s="0" t="inlineStr">
+        <is>
+          <t>sequence</t>
+        </is>
+      </c>
+      <c r="L101" s="0" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="M101" s="0" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="N101" s="0" t="inlineStr">
+        <is>
+          <t>章节内顺序</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="J102" s="0" t="inlineStr">
+        <is>
+          <t>speaker</t>
+        </is>
+      </c>
+      <c r="L102" s="0" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="M102" s="0" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="N102" s="0" t="inlineStr">
+        <is>
+          <t>说话人，空表示旁白</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="J103" s="0" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="L103" s="0" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="M103" s="0" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="N103" s="0" t="inlineStr">
+        <is>
+          <t>文本内容</t>
         </is>
       </c>
     </row>

</xml_diff>